<commit_message>
Atualização automática: Dispersão KM por Motorista.xlsx
</commit_message>
<xml_diff>
--- a/Dispersão KM por Motorista.xlsx
+++ b/Dispersão KM por Motorista.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" r:id="R0963e7c0761c46bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" r:id="R07ca969c74884015"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -99,7 +99,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.22186495176848875</x:v>
+        <x:v>0.33404947160608534</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -130,6 +130,19 @@
     </x:row>
     <x:row>
       <x:c s="8">
+        <x:v>1265</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>APARECIDO  LIMA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.13177750482540795</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
         <x:v>10</x:v>
       </x:c>
       <x:c t="inlineStr">
@@ -151,7 +164,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.15390847434087185</x:v>
+        <x:v>0.12705549054628329</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -169,6 +182,32 @@
     </x:row>
     <x:row>
       <x:c s="8">
+        <x:v>694</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>DILSON  FRANCA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.43706640237859262</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>294</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>EDENILSON  FAZAN</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.1718983557548579</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
         <x:v>118</x:v>
       </x:c>
       <x:c t="inlineStr">
@@ -203,7 +242,20 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.46249832282302417</x:v>
+        <x:v>0.40241879542781311</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>EVERTON  ARAUJO</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.388235294117647</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -216,7 +268,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.41816966027081737</x:v>
+        <x:v>0.3627471810915166</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -242,7 +294,20 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.17338273892234057</x:v>
+        <x:v>0.20692611006343231</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>GEOVANE  SILVA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.018990273274664293</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -255,7 +320,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.11487027735107591</x:v>
+        <x:v>0.19296604105894666</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -281,7 +346,20 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.17507720164200746</x:v>
+        <x:v>0.18729351417144824</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>IGOR  ARAUJO</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.18893642423639445</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -320,7 +398,20 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.35085276299972645</x:v>
+        <x:v>0.32228038012239746</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>553</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>JHONATAN  RODRIGUES</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.46801051709027175</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -333,7 +424,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.1787085159142634</x:v>
+        <x:v>0.16312713384642086</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -351,6 +442,19 @@
     </x:row>
     <x:row>
       <x:c s="8">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>JORGE  LIMA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.15929239038870402</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
         <x:v>323</x:v>
       </x:c>
       <x:c t="inlineStr">
@@ -364,6 +468,32 @@
     </x:row>
     <x:row>
       <x:c s="8">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>JOSE  RODRIGUES</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.066721021877972575</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>246</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>JOSE  SOUZA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.37777296159264351</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
         <x:v>453</x:v>
       </x:c>
       <x:c t="inlineStr">
@@ -424,7 +554,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.24234912653751728</x:v>
+        <x:v>0.21016866556569314</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -489,7 +619,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.21293609794069779</x:v>
+        <x:v>0.23599182442907796</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -502,7 +632,20 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.12342259156663582</x:v>
+        <x:v>0.11427034503957567</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>341</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>NILDO  TONIAZZO</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.11943149690532584</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -520,6 +663,19 @@
     </x:row>
     <x:row>
       <x:c s="8">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>PODALIRIO  NATES</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.36116876896056205</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
         <x:v>16</x:v>
       </x:c>
       <x:c t="inlineStr">
@@ -528,7 +684,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.8369095292172215</x:v>
+        <x:v>0.53267663214919625</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -546,6 +702,19 @@
     </x:row>
     <x:row>
       <x:c s="8">
+        <x:v>320</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>RENAN  ARAUJO</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.10073736141318768</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
         <x:v>287</x:v>
       </x:c>
       <x:c t="inlineStr">
@@ -554,7 +723,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.13083680658769348</x:v>
+        <x:v>0.16335386406665053</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -567,7 +736,33 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.48863719134678418</x:v>
+        <x:v>0.44319699928064948</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>348</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>STEFANES  TERNOSKI</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.96850393700787407</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>TENISON  RODRIGUES</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.025923330997897898</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -594,6 +789,19 @@
       </x:c>
       <x:c s="9">
         <x:v>0.741620868488273</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>VINALDO  SOUZA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.40717203812982294</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -630,7 +838,7 @@
       </x:c>
       <x:c s="1"/>
       <x:c s="10">
-        <x:v>0.25160836450567992</x:v>
+        <x:v>0.24598136659993819</x:v>
       </x:c>
     </x:row>
     <x:row/>
@@ -640,9 +848,8 @@
           <x:t>Filtros aplicados:
 Mapas KM maior que 0
 Revenda é GranDourados
-Frota é Padronizada
 Ano é 2026
-Date é igual a ou está depois de 01/09/2026 e está antes de 11/09/2026
+Date é igual a ou está depois de 01/09/2026 e está antes de 13/09/2026
 Taxa de Dispersão é Até 100%
 Check Dispersão KM é Sim
 Tipo Dispersão KM é Positiva

</xml_diff>